<commit_message>
Remove N/A so columns are properly numbers
</commit_message>
<xml_diff>
--- a/data/Battery Test Results 2025-2026 Season.xlsx
+++ b/data/Battery Test Results 2025-2026 Season.xlsx
@@ -18,25 +18,25 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={09c085d8-224a-4c9e-81a4-dd66d5c001f9}</author>
-    <author>tc={2d2cfd80-111f-4df7-8aab-665a51fba5a3}</author>
+    <author>tc={6a11a031-710a-4d72-ae58-62e7028d80bb}</author>
+    <author>tc={9ee4eab9-2351-4e9b-bcd6-83985e65f4ba}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{09c085d8-224a-4c9e-81a4-dd66d5c001f9}" ref="A1">
+    <comment authorId="0" xr:uid="{6a11a031-710a-4d72-ae58-62e7028d80bb}" ref="A1">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Outlier?
+</t>
+      </text>
+    </comment>
+    <comment authorId="1" xr:uid="{9ee4eab9-2351-4e9b-bcd6-83985e65f4ba}" ref="A1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
 	Charging
-</t>
-      </text>
-    </comment>
-    <comment authorId="1" xr:uid="{2d2cfd80-111f-4df7-8aab-665a51fba5a3}" ref="A1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Outlier?
 </t>
       </text>
     </comment>
@@ -47,10 +47,10 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={ee7a26a1-c149-4ee7-9232-e45df0033c96}</author>
+    <author>tc={64e1ec64-a0bc-4eae-a0ea-f941be5bc2e6}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{ee7a26a1-c149-4ee7-9232-e45df0033c96}" ref="B39">
+    <comment authorId="0" xr:uid="{64e1ec64-a0bc-4eae-a0ea-f941be5bc2e6}" ref="B39">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="113">
   <si>
     <t>Battery</t>
   </si>
@@ -327,16 +327,22 @@
     <t>2026mnwi_f1m1</t>
   </si>
   <si>
-    <t>N/A</t>
+    <t>voltage after not recorded?</t>
   </si>
   <si>
     <t>2026mnwi_f1m2</t>
+  </si>
+  <si>
+    <t>no data recorded?</t>
   </si>
   <si>
     <t>Battery Name</t>
   </si>
   <si>
     <t>Capacity Ah / Wh</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
   <si>
     <t>Very Jumpy @ Beginning</t>
@@ -1174,11 +1180,11 @@
           </c:val>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="884057816"/>
-        <c:axId val="2026230060"/>
+        <c:axId val="1044438935"/>
+        <c:axId val="695971764"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="884057816"/>
+        <c:axId val="1044438935"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1230,10 +1236,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2026230060"/>
+        <c:crossAx val="695971764"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2026230060"/>
+        <c:axId val="695971764"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1308,7 +1314,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="884057816"/>
+        <c:crossAx val="1044438935"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1394,7 +1400,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="David Chen" id="{ec2e362d-0493-403c-9f1d-f9d021c2d2f4}" providerId="google-sheets"/>
+  <x18tc:person displayName="David Chen" id="{b05be591-982a-4678-a2b9-85ae104c8f98}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -1594,10 +1600,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A1" dT="2026-01-16T01:46:15.00" personId="{ec2e362d-0493-403c-9f1d-f9d021c2d2f4}" id="{09c085d8-224a-4c9e-81a4-dd66d5c001f9}" done="0">
+  <x18tc:threadedComment ref="A1" dT="2026-01-16T01:46:15.00" personId="{b05be591-982a-4678-a2b9-85ae104c8f98}" id="{9ee4eab9-2351-4e9b-bcd6-83985e65f4ba}" done="0">
     <x18tc:text xml:space="preserve">Charging</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-02-03T23:55:01.00" personId="{ec2e362d-0493-403c-9f1d-f9d021c2d2f4}" id="{2d2cfd80-111f-4df7-8aab-665a51fba5a3}" done="0">
+  <x18tc:threadedComment ref="A1" dT="2026-02-03T23:55:01.00" personId="{b05be591-982a-4678-a2b9-85ae104c8f98}" id="{6a11a031-710a-4d72-ae58-62e7028d80bb}" done="0">
     <x18tc:text xml:space="preserve">Outlier?</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1605,7 +1611,7 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="B39" dT="2026-02-03T23:55:28.00" personId="{ec2e362d-0493-403c-9f1d-f9d021c2d2f4}" id="{ee7a26a1-c149-4ee7-9232-e45df0033c96}" done="1">
+  <x18tc:threadedComment ref="B39" dT="2026-02-03T23:55:28.00" personId="{b05be591-982a-4678-a2b9-85ae104c8f98}" id="{64e1ec64-a0bc-4eae-a0ea-f941be5bc2e6}" done="1">
     <x18tc:text xml:space="preserve">Outlier?</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -9988,11 +9994,12 @@
       <c r="D18" s="44">
         <v>13.237</v>
       </c>
-      <c r="E18" s="44" t="s">
-        <v>87</v>
-      </c>
+      <c r="E18" s="41"/>
       <c r="F18" s="44" t="s">
         <v>70</v>
+      </c>
+      <c r="G18" s="44" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="19">
@@ -10002,17 +10009,14 @@
       <c r="B19" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="D19" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="E19" s="44" t="s">
-        <v>87</v>
-      </c>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
       <c r="F19" s="44" t="s">
         <v>70</v>
+      </c>
+      <c r="G19" s="44" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="20">
@@ -16915,14 +16919,14 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="45" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="45" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E1" s="47"/>
       <c r="F1" s="45" t="s">
@@ -17173,7 +17177,7 @@
         <v>62.619</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="H9" s="12">
         <v>13.091</v>
@@ -17273,10 +17277,10 @@
         <v>20.0</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="J12" s="16"/>
       <c r="K12" s="17"/>
@@ -17830,7 +17834,7 @@
         <v>13.399</v>
       </c>
       <c r="I33" s="15" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="J33" s="16"/>
       <c r="K33" s="17"/>
@@ -18254,10 +18258,10 @@
         <v>17.0</v>
       </c>
       <c r="H49" s="15" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I49" s="15" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="J49" s="26"/>
       <c r="K49" s="27"/>
@@ -18722,13 +18726,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E1" s="52"/>
       <c r="F1" s="1" t="s">
@@ -19430,7 +19434,7 @@
         <v>12.785</v>
       </c>
       <c r="J23" s="26" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -19498,16 +19502,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="44" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C1" s="44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D1" s="44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E1" s="44" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2">
@@ -19515,10 +19519,10 @@
         <v>45</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3">
@@ -19526,10 +19530,10 @@
         <v>11</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C3" s="44" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4">
@@ -19537,10 +19541,10 @@
         <v>8</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5">
@@ -19548,10 +19552,10 @@
         <v>13</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C5" s="44" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6">
@@ -19559,10 +19563,10 @@
         <v>10</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7">
@@ -19570,10 +19574,10 @@
         <v>9</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C7" s="44" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8">
@@ -19581,10 +19585,10 @@
         <v>14</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9">
@@ -19592,10 +19596,10 @@
         <v>16</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C9" s="44" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10">
@@ -19603,10 +19607,10 @@
         <v>17</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11">
@@ -19614,7 +19618,7 @@
         <v>35</v>
       </c>
       <c r="B11" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C11" s="44" t="s">
         <v>70</v>
@@ -19625,10 +19629,10 @@
         <v>47</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C12" s="44" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13">
@@ -19636,7 +19640,7 @@
         <v>43</v>
       </c>
       <c r="B13" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C13" s="44" t="s">
         <v>70</v>
@@ -19647,7 +19651,7 @@
         <v>49</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C14" s="44" t="s">
         <v>70</v>
@@ -19658,7 +19662,7 @@
         <v>37</v>
       </c>
       <c r="B15" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C15" s="44" t="s">
         <v>70</v>
@@ -19669,7 +19673,7 @@
         <v>53</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C16" s="44" t="s">
         <v>70</v>
@@ -19680,7 +19684,7 @@
         <v>42</v>
       </c>
       <c r="B17" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C17" s="44" t="s">
         <v>70</v>
@@ -19691,7 +19695,7 @@
         <v>55</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C18" s="44" t="s">
         <v>70</v>
@@ -19702,7 +19706,7 @@
         <v>38</v>
       </c>
       <c r="B19" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C19" s="44" t="s">
         <v>70</v>
@@ -19713,7 +19717,7 @@
         <v>40</v>
       </c>
       <c r="B20" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C20" s="44" t="s">
         <v>70</v>
@@ -19724,7 +19728,7 @@
         <v>51</v>
       </c>
       <c r="B21" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C21" s="44" t="s">
         <v>70</v>
@@ -19744,20 +19748,20 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="60" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B1" s="61" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C1" s="62"/>
       <c r="D1" s="63" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E1" s="63" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F1" s="63" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G1" s="63" t="s">
         <v>5</v>
@@ -19766,7 +19770,7 @@
         <v>6</v>
       </c>
       <c r="I1" s="65" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J1" s="66"/>
       <c r="K1" s="61" t="s">
@@ -19821,7 +19825,7 @@
         <v>12.738</v>
       </c>
       <c r="I2" s="71" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K2" s="41">
         <f>IFERROR(__xludf.DUMMYFUNCTION("ROUND(AVERAGE(FILTER($D:$D, $B:$B = K1)), 2)"),5.97)</f>
@@ -19878,7 +19882,7 @@
       <c r="G3" s="69"/>
       <c r="H3" s="70"/>
       <c r="I3" s="71" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="K3" s="41">
         <f>IFERROR(__xludf.DUMMYFUNCTION("ROUND(AVERAGE(FILTER($E:$E, $B:$B = K1)), 2)"),77.66)</f>
@@ -19939,7 +19943,7 @@
         <v>12.595</v>
       </c>
       <c r="I4" s="71" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K4" s="41">
         <f>IFERROR(__xludf.DUMMYFUNCTION("ROUND(AVERAGE(FILTER($F:$F, $B:$B = K1)), 2)"),16.2)</f>
@@ -20000,7 +20004,7 @@
         <v>13.116</v>
       </c>
       <c r="I5" s="71" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K5" s="41">
         <f>IFERROR(__xludf.DUMMYFUNCTION("ROUND(AVERAGE(FILTER($G:$G, $B:$B = K1)), 2)"),13.27)</f>
@@ -20059,7 +20063,7 @@
       </c>
       <c r="H6" s="70"/>
       <c r="I6" s="71" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K6" s="41">
         <f>IFERROR(__xludf.DUMMYFUNCTION("ROUND(AVERAGE(FILTER($H:$H, $B:$B = K1)), 2)"),12.95)</f>
@@ -20121,7 +20125,7 @@
       </c>
       <c r="I7" s="73"/>
       <c r="J7" s="44" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="K7" s="61" t="s">
         <v>11</v>
@@ -20174,7 +20178,7 @@
       </c>
       <c r="I8" s="73"/>
       <c r="J8" s="44" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K8" s="74">
         <f t="shared" ref="K8:S8" si="1">(K2-min($K2:$S2))/(max($K2:$S2)-min($K2:$S2))</f>
@@ -20236,7 +20240,7 @@
       </c>
       <c r="I9" s="73"/>
       <c r="J9" s="44" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="K9" s="74">
         <f t="shared" ref="K9:S9" si="2">(K3-min($K3:$S3))/(max($K3:$S3)-min($K3:$S3))</f>
@@ -20332,7 +20336,7 @@
       </c>
       <c r="I11" s="73"/>
       <c r="J11" s="44" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K11" s="74">
         <f t="shared" ref="K11:S11" si="3">1-(K4-min($K4:$S4))/(max($K4:$S4)-min($K4:$S4))</f>

</xml_diff>